<commit_message>
docs(spec): complete the loops review checklist and update the prompts sheet
</commit_message>
<xml_diff>
--- a/specs/claude-loops/prompts.xlsx
+++ b/specs/claude-loops/prompts.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="48">
   <si>
     <t xml:space="preserve">Session</t>
   </si>
@@ -36,7 +36,7 @@
 Start to plan implementation for loops.</t>
   </si>
   <si>
-    <t xml:space="preserve">-</t>
+    <t xml:space="preserve">Chatgpt</t>
   </si>
   <si>
     <t xml:space="preserve">The following is main prompt for claude I want to split it to pass to speckit commands and where should I pass description file:
@@ -156,40 +156,10 @@
 The development loops SHOULD be validated against the reference application as an end-to-end demonstration that they can consume real project requirements and produce a working application.</t>
   </si>
   <si>
-    <t xml:space="preserve">/speckit-specify Read the task description at: @specs/claude-loops/task-description.md
-Create the specification for Goal #1 only: implementing the reusable development loops.
-The scope of this specification is limited to the reusable development-loop infrastructure:
-- backend-dev
-- frontend-dev
-- shared loop functionality
-- optional orchestration between the loops
-Do NOT specify, design, implement, or decompose the application described by the PRD.
-The application/PRD is only contextual information about how the reusable loops will eventually be used. Its application-specific requirements are out of scope for this specification.
-The task description is the primary source of requirements. Do not invent requirements that are not supported by the task description or the repository constitution.
-The specification should describe:
-- What each loop does
-- Their supported inputs
-- Their expected outputs and artifacts
-- Their iteration behavior
-- How they determine the next unit of work
-- How they verify implementation
-- Completion and stopping conditions
-- Failure and retry handling
-- Validation behavior
-- State and progress tracking
-- Safeguards against uncontrolled or unrelated changes
-- Shared behavior and functionality between the loops
-- How the loops interact with Claude Code
-- How the loops can be executed independently
-- How they may be used through an orchestrator
-- Expected user/developer workflow
-- Reusability across different applications and PRDs/User Stories
-Clearly distinguish between:
-- Explicitly required behavior from the task description.
-- Behavior reasonably implied by the task description.
-- Unresolved questions and ambiguities.
-Do not silently convert assumptions or recommendations into requirements.
-Do not work on the application described by the PRD.</t>
+    <t xml:space="preserve">Opus 5.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">apply them</t>
   </si>
   <si>
     <t xml:space="preserve">/speckit-clarify Review the current Claude Loops specification against the authoritative task description:
@@ -371,6 +341,93 @@
   <si>
     <t xml:space="preserve">Apply your recommendations for top 4 issues</t>
   </si>
+  <si>
+    <t xml:space="preserve">71d6118c-1fc5-4a40-975d-d468fb0a92bb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement Phase 1: T001-T007</t>
+  </si>
+  <si>
+    <t xml:space="preserve">before continue I want to rename from claude-loops to claude-dev-loops or suggest a valid name for this project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Add in .gitignore all possible ignore files for this project, then commit all changes but phase 1 impl in a separate commit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T008-T019</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T020-T027</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/code-review</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yes, fix all three with tests</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commit phase 2 impl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">60d3a0f2-3a08-4103-bcf9-ab92592d3c29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">speckit-implement T028-T030</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sonnet 5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T031-T037</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a6ade60a-3b28-4dbb-abba-d7f80e640103</t>
+  </si>
+  <si>
+    <t xml:space="preserve">327d459d-3ef3-4316-9689-d26f4cb14524</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0ff13f96-fdec-4494-a914-43950b8f559d</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement Phase 4: T038-T046</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fix all seven, check UI-origin requests for #6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commit phase 3 and 4 impl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T047-T050</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T051-T056</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19246cf3-3402-4e12-8fb8-9e1c0e715583</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T057-T063</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement continue phase 7 T063-T066</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement Phase 8: T067-T069</t>
+  </si>
+  <si>
+    <t xml:space="preserve">go ahead with apply fix</t>
+  </si>
+  <si>
+    <t xml:space="preserve">commit phase 8 and 9 impl</t>
+  </si>
+  <si>
+    <t xml:space="preserve">/speckit-implement T076</t>
+  </si>
+  <si>
+    <t xml:space="preserve">-</t>
+  </si>
 </sst>
 </file>
 
@@ -384,6 +441,7 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -406,6 +464,7 @@
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -456,16 +515,20 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -592,188 +655,619 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C1048576"/>
+  <dimension ref="A1:F1048576"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="17" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="35.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="47.72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="47.72"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="true" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" s="2" customFormat="true" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="2" t="s">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>3</v>
+      <c r="C4" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="0" t="s">
-        <v>3</v>
+      <c r="A5" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="s">
+      <c r="A6" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B38" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="C6" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B11" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B12" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B13" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="C13" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B14" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="C14" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B15" s="0" t="s">
-        <v>15</v>
-      </c>
-      <c r="C15" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
-        <v>5</v>
-      </c>
-      <c r="B16" s="0" t="s">
-        <v>17</v>
-      </c>
-      <c r="C16" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C17" s="0" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C18" s="0" t="s">
-        <v>3</v>
+      <c r="C38" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C47" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C48" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C49" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C50" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C51" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C52" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C53" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C54" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C55" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C56" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C57" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C58" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C59" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C60" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C61" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C62" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C63" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C64" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C65" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C66" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="17" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C67" s="1" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>

</xml_diff>